<commit_message>
Altura normal, columnas compactas y bordes grises en Excel
</commit_message>
<xml_diff>
--- a/site/assets/docs/ficha-medicion-antena-rufcom.xlsx
+++ b/site/assets/docs/ficha-medicion-antena-rufcom.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi prueba" sheetId="1" r:id="R4c047fd2658e494d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo y ayuda" sheetId="2" r:id="Rc14d970cfa7b4743"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi prueba" sheetId="1" r:id="Rce631ae0a75a4d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo y ayuda" sheetId="2" r:id="R546b752d338545fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +60,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -68,22 +68,18 @@
       </x:bottom>
     </x:border>
     <x:border>
-      <x:bottom style="thin">
-        <x:color rgb="FFE7E7E7"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0D0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0D0"/>
+      </x:right>
       <x:top style="thin">
-        <x:color rgb="FFE7E7E7"/>
+        <x:color rgb="FFD0D0D0"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFE7E7E7"/>
+        <x:color rgb="FFD0D0D0"/>
       </x:bottom>
-    </x:border>
-    <x:border>
-      <x:top style="thin">
-        <x:color rgb="FFE7E7E7"/>
-      </x:top>
     </x:border>
     <x:border>
       <x:top style="thin">
@@ -97,7 +93,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -134,6 +130,9 @@
     <x:xf numFmtId="202" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -143,23 +142,14 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -167,7 +157,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -207,13 +197,13 @@
     <xdr:ext cx="1714500" cy="571500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b49f22c5-fafe-4749-ad16-e36eabcf08d2"/>
+        <xdr:cNvPr id="1" name="06bcd0a7-42ad-4d4c-bb28-a4132ee9dc48"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6a8c5202da194438"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R151702c94ea04d54"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -239,13 +229,13 @@
     <xdr:ext cx="1714500" cy="571500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="16cda0aa-6784-488d-a6e4-60b0161f54bd"/>
+        <xdr:cNvPr id="1" name="07887ead-9b31-42a0-9194-560e70820e46"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3a00e68b55fe44ba"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb95473afedce489e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -472,10 +462,10 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="31" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
   </x:cols>
@@ -569,50 +559,50 @@
         <x:v>Fecha de la prueba</x:v>
       </x:c>
       <x:c r="B10" s="6"/>
-      <x:c r="C10" s="23" t="str"/>
-      <x:c r="D10" s="24"/>
-      <x:c r="E10" s="24"/>
-      <x:c r="F10" s="24"/>
+      <x:c r="C10" s="21" t="str"/>
+      <x:c r="D10" s="22"/>
+      <x:c r="E10" s="22"/>
+      <x:c r="F10" s="22"/>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>Antena que probé</x:v>
       </x:c>
       <x:c r="B11" s="6"/>
-      <x:c r="C11" s="25" t="str"/>
-      <x:c r="D11" s="25"/>
-      <x:c r="E11" s="25"/>
-      <x:c r="F11" s="25"/>
+      <x:c r="C11" s="23" t="str"/>
+      <x:c r="D11" s="23"/>
+      <x:c r="E11" s="23"/>
+      <x:c r="F11" s="23"/>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>Instrumento usado</x:v>
       </x:c>
       <x:c r="B12" s="6"/>
-      <x:c r="C12" s="25" t="str"/>
-      <x:c r="D12" s="25"/>
-      <x:c r="E12" s="25"/>
-      <x:c r="F12" s="25"/>
+      <x:c r="C12" s="23" t="str"/>
+      <x:c r="D12" s="23"/>
+      <x:c r="E12" s="23"/>
+      <x:c r="F12" s="23"/>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>Dónde medí</x:v>
       </x:c>
       <x:c r="B13" s="6"/>
-      <x:c r="C13" s="25" t="str"/>
-      <x:c r="D13" s="25"/>
-      <x:c r="E13" s="25"/>
-      <x:c r="F13" s="25"/>
+      <x:c r="C13" s="23" t="str"/>
+      <x:c r="D13" s="23"/>
+      <x:c r="E13" s="23"/>
+      <x:c r="F13" s="23"/>
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>Montaje y lugar</x:v>
       </x:c>
       <x:c r="B14" s="6"/>
-      <x:c r="C14" s="25" t="str"/>
-      <x:c r="D14" s="25"/>
-      <x:c r="E14" s="25"/>
-      <x:c r="F14" s="25"/>
+      <x:c r="C14" s="23" t="str"/>
+      <x:c r="D14" s="23"/>
+      <x:c r="E14" s="23"/>
+      <x:c r="F14" s="23"/>
     </x:row>
     <x:row r="15" ht="8" customHeight="1">
       <x:c r="A15" s="3"/>
@@ -651,424 +641,424 @@
       <x:c r="F18" s="3"/>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
-      <x:c r="A19" s="11" t="str">
+      <x:c r="A19" s="14" t="str">
         <x:v>Frecuencia (MHz)</x:v>
       </x:c>
-      <x:c r="B19" s="11" t="str">
+      <x:c r="B19" s="14" t="str">
         <x:v>ROE leída</x:v>
       </x:c>
-      <x:c r="C19" s="11" t="str">
+      <x:c r="C19" s="14" t="str">
         <x:v>Cable (metros)</x:v>
       </x:c>
-      <x:c r="D19" s="11" t="str">
+      <x:c r="D19" s="14" t="str">
         <x:v>Potencia (W; opcional)</x:v>
       </x:c>
-      <x:c r="E19" s="11" t="str">
+      <x:c r="E19" s="14" t="str">
         <x:v>Qué cambié entre lecturas</x:v>
       </x:c>
-      <x:c r="F19" s="11" t="str">
+      <x:c r="F19" s="14" t="str">
         <x:v>Foto o nota (opcional)</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="28" customHeight="1">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="15"/>
-      <x:c r="C20" s="15"/>
-      <x:c r="D20" s="15"/>
-      <x:c r="E20" s="16"/>
-      <x:c r="F20" s="16"/>
-    </x:row>
-    <x:row r="21" ht="28" customHeight="1">
-      <x:c r="A21" s="17"/>
-      <x:c r="B21" s="18"/>
-      <x:c r="C21" s="18"/>
-      <x:c r="D21" s="18"/>
-      <x:c r="E21" s="19"/>
-      <x:c r="F21" s="19"/>
-    </x:row>
-    <x:row r="22" ht="28" customHeight="1">
-      <x:c r="A22" s="17"/>
-      <x:c r="B22" s="18"/>
-      <x:c r="C22" s="18"/>
-      <x:c r="D22" s="18"/>
-      <x:c r="E22" s="19"/>
-      <x:c r="F22" s="19"/>
-    </x:row>
-    <x:row r="23" ht="28" customHeight="1">
-      <x:c r="A23" s="17"/>
-      <x:c r="B23" s="18"/>
-      <x:c r="C23" s="18"/>
-      <x:c r="D23" s="18"/>
-      <x:c r="E23" s="19"/>
-      <x:c r="F23" s="19"/>
-    </x:row>
-    <x:row r="24" ht="28" customHeight="1">
-      <x:c r="A24" s="17"/>
-      <x:c r="B24" s="18"/>
-      <x:c r="C24" s="18"/>
-      <x:c r="D24" s="18"/>
-      <x:c r="E24" s="19"/>
-      <x:c r="F24" s="19"/>
-    </x:row>
-    <x:row r="25" ht="28" customHeight="1">
-      <x:c r="A25" s="17"/>
-      <x:c r="B25" s="18"/>
-      <x:c r="C25" s="18"/>
-      <x:c r="D25" s="18"/>
-      <x:c r="E25" s="19"/>
-      <x:c r="F25" s="19"/>
-    </x:row>
-    <x:row r="26" ht="28" customHeight="1">
-      <x:c r="A26" s="17"/>
-      <x:c r="B26" s="18"/>
-      <x:c r="C26" s="18"/>
-      <x:c r="D26" s="18"/>
-      <x:c r="E26" s="19"/>
-      <x:c r="F26" s="19"/>
-    </x:row>
-    <x:row r="27" ht="28" customHeight="1">
-      <x:c r="A27" s="17"/>
-      <x:c r="B27" s="18"/>
-      <x:c r="C27" s="18"/>
-      <x:c r="D27" s="18"/>
-      <x:c r="E27" s="19"/>
-      <x:c r="F27" s="19"/>
-    </x:row>
-    <x:row r="28" ht="28" customHeight="1">
-      <x:c r="A28" s="17"/>
-      <x:c r="B28" s="18"/>
-      <x:c r="C28" s="18"/>
-      <x:c r="D28" s="18"/>
-      <x:c r="E28" s="19"/>
-      <x:c r="F28" s="19"/>
-    </x:row>
-    <x:row r="29" ht="28" customHeight="1">
-      <x:c r="A29" s="17"/>
-      <x:c r="B29" s="18"/>
-      <x:c r="C29" s="18"/>
-      <x:c r="D29" s="18"/>
-      <x:c r="E29" s="19"/>
-      <x:c r="F29" s="19"/>
-    </x:row>
-    <x:row r="30" ht="28" customHeight="1">
-      <x:c r="A30" s="17"/>
-      <x:c r="B30" s="18"/>
-      <x:c r="C30" s="18"/>
-      <x:c r="D30" s="18"/>
-      <x:c r="E30" s="19"/>
-      <x:c r="F30" s="19"/>
-    </x:row>
-    <x:row r="31" ht="28" customHeight="1">
-      <x:c r="A31" s="17"/>
-      <x:c r="B31" s="18"/>
-      <x:c r="C31" s="18"/>
-      <x:c r="D31" s="18"/>
-      <x:c r="E31" s="19"/>
-      <x:c r="F31" s="19"/>
-    </x:row>
-    <x:row r="32" ht="28" customHeight="1">
-      <x:c r="A32" s="17"/>
-      <x:c r="B32" s="18"/>
-      <x:c r="C32" s="18"/>
-      <x:c r="D32" s="18"/>
-      <x:c r="E32" s="19"/>
-      <x:c r="F32" s="19"/>
-    </x:row>
-    <x:row r="33" ht="28" customHeight="1">
-      <x:c r="A33" s="17"/>
-      <x:c r="B33" s="18"/>
-      <x:c r="C33" s="18"/>
-      <x:c r="D33" s="18"/>
-      <x:c r="E33" s="19"/>
-      <x:c r="F33" s="19"/>
-    </x:row>
-    <x:row r="34" ht="28" customHeight="1">
-      <x:c r="A34" s="17"/>
-      <x:c r="B34" s="18"/>
-      <x:c r="C34" s="18"/>
-      <x:c r="D34" s="18"/>
-      <x:c r="E34" s="19"/>
-      <x:c r="F34" s="19"/>
-    </x:row>
-    <x:row r="35" ht="28" customHeight="1">
-      <x:c r="A35" s="17"/>
-      <x:c r="B35" s="18"/>
-      <x:c r="C35" s="18"/>
-      <x:c r="D35" s="18"/>
-      <x:c r="E35" s="19"/>
-      <x:c r="F35" s="19"/>
-    </x:row>
-    <x:row r="36" ht="28" customHeight="1">
-      <x:c r="A36" s="17"/>
-      <x:c r="B36" s="18"/>
-      <x:c r="C36" s="18"/>
-      <x:c r="D36" s="18"/>
-      <x:c r="E36" s="19"/>
-      <x:c r="F36" s="19"/>
-    </x:row>
-    <x:row r="37" ht="28" customHeight="1">
-      <x:c r="A37" s="17"/>
-      <x:c r="B37" s="18"/>
-      <x:c r="C37" s="18"/>
-      <x:c r="D37" s="18"/>
-      <x:c r="E37" s="19"/>
-      <x:c r="F37" s="19"/>
-    </x:row>
-    <x:row r="38" ht="28" customHeight="1">
-      <x:c r="A38" s="17"/>
-      <x:c r="B38" s="18"/>
-      <x:c r="C38" s="18"/>
-      <x:c r="D38" s="18"/>
-      <x:c r="E38" s="19"/>
-      <x:c r="F38" s="19"/>
-    </x:row>
-    <x:row r="39" ht="28" customHeight="1">
-      <x:c r="A39" s="17"/>
-      <x:c r="B39" s="18"/>
-      <x:c r="C39" s="18"/>
-      <x:c r="D39" s="18"/>
-      <x:c r="E39" s="19"/>
-      <x:c r="F39" s="19"/>
-    </x:row>
-    <x:row r="40" ht="28" customHeight="1">
-      <x:c r="A40" s="17"/>
-      <x:c r="B40" s="18"/>
-      <x:c r="C40" s="18"/>
-      <x:c r="D40" s="18"/>
-      <x:c r="E40" s="19"/>
-      <x:c r="F40" s="19"/>
-    </x:row>
-    <x:row r="41" ht="28" customHeight="1">
-      <x:c r="A41" s="17"/>
-      <x:c r="B41" s="18"/>
-      <x:c r="C41" s="18"/>
-      <x:c r="D41" s="18"/>
-      <x:c r="E41" s="19"/>
-      <x:c r="F41" s="19"/>
-    </x:row>
-    <x:row r="42" ht="28" customHeight="1">
-      <x:c r="A42" s="17"/>
-      <x:c r="B42" s="18"/>
-      <x:c r="C42" s="18"/>
-      <x:c r="D42" s="18"/>
-      <x:c r="E42" s="19"/>
-      <x:c r="F42" s="19"/>
-    </x:row>
-    <x:row r="43" ht="28" customHeight="1">
-      <x:c r="A43" s="17"/>
-      <x:c r="B43" s="18"/>
-      <x:c r="C43" s="18"/>
-      <x:c r="D43" s="18"/>
-      <x:c r="E43" s="19"/>
-      <x:c r="F43" s="19"/>
-    </x:row>
-    <x:row r="44" ht="28" customHeight="1">
-      <x:c r="A44" s="17"/>
-      <x:c r="B44" s="18"/>
-      <x:c r="C44" s="18"/>
-      <x:c r="D44" s="18"/>
-      <x:c r="E44" s="19"/>
-      <x:c r="F44" s="19"/>
-    </x:row>
-    <x:row r="45" ht="28" customHeight="1">
-      <x:c r="A45" s="17"/>
-      <x:c r="B45" s="18"/>
-      <x:c r="C45" s="18"/>
-      <x:c r="D45" s="18"/>
-      <x:c r="E45" s="19"/>
-      <x:c r="F45" s="19"/>
-    </x:row>
-    <x:row r="46" ht="28" customHeight="1">
-      <x:c r="A46" s="17"/>
-      <x:c r="B46" s="18"/>
-      <x:c r="C46" s="18"/>
-      <x:c r="D46" s="18"/>
-      <x:c r="E46" s="19"/>
-      <x:c r="F46" s="19"/>
-    </x:row>
-    <x:row r="47" ht="28" customHeight="1">
-      <x:c r="A47" s="17"/>
-      <x:c r="B47" s="18"/>
-      <x:c r="C47" s="18"/>
-      <x:c r="D47" s="18"/>
-      <x:c r="E47" s="19"/>
-      <x:c r="F47" s="19"/>
-    </x:row>
-    <x:row r="48" ht="28" customHeight="1">
-      <x:c r="A48" s="17"/>
-      <x:c r="B48" s="18"/>
-      <x:c r="C48" s="18"/>
-      <x:c r="D48" s="18"/>
-      <x:c r="E48" s="19"/>
-      <x:c r="F48" s="19"/>
-    </x:row>
-    <x:row r="49" ht="28" customHeight="1">
-      <x:c r="A49" s="17"/>
-      <x:c r="B49" s="18"/>
-      <x:c r="C49" s="18"/>
-      <x:c r="D49" s="18"/>
-      <x:c r="E49" s="19"/>
-      <x:c r="F49" s="19"/>
-    </x:row>
-    <x:row r="50" ht="28" customHeight="1">
-      <x:c r="A50" s="17"/>
-      <x:c r="B50" s="18"/>
-      <x:c r="C50" s="18"/>
-      <x:c r="D50" s="18"/>
-      <x:c r="E50" s="19"/>
-      <x:c r="F50" s="19"/>
-    </x:row>
-    <x:row r="51" ht="28" customHeight="1">
-      <x:c r="A51" s="17"/>
-      <x:c r="B51" s="18"/>
-      <x:c r="C51" s="18"/>
-      <x:c r="D51" s="18"/>
-      <x:c r="E51" s="19"/>
-      <x:c r="F51" s="19"/>
-    </x:row>
-    <x:row r="52" ht="28" customHeight="1">
-      <x:c r="A52" s="17"/>
-      <x:c r="B52" s="18"/>
-      <x:c r="C52" s="18"/>
-      <x:c r="D52" s="18"/>
-      <x:c r="E52" s="19"/>
-      <x:c r="F52" s="19"/>
-    </x:row>
-    <x:row r="53" ht="28" customHeight="1">
-      <x:c r="A53" s="17"/>
-      <x:c r="B53" s="18"/>
-      <x:c r="C53" s="18"/>
-      <x:c r="D53" s="18"/>
-      <x:c r="E53" s="19"/>
-      <x:c r="F53" s="19"/>
-    </x:row>
-    <x:row r="54" ht="28" customHeight="1">
-      <x:c r="A54" s="17"/>
-      <x:c r="B54" s="18"/>
-      <x:c r="C54" s="18"/>
-      <x:c r="D54" s="18"/>
-      <x:c r="E54" s="19"/>
-      <x:c r="F54" s="19"/>
-    </x:row>
-    <x:row r="55" ht="28" customHeight="1">
-      <x:c r="A55" s="17"/>
-      <x:c r="B55" s="18"/>
-      <x:c r="C55" s="18"/>
-      <x:c r="D55" s="18"/>
-      <x:c r="E55" s="19"/>
-      <x:c r="F55" s="19"/>
-    </x:row>
-    <x:row r="56" ht="28" customHeight="1">
-      <x:c r="A56" s="17"/>
-      <x:c r="B56" s="18"/>
-      <x:c r="C56" s="18"/>
-      <x:c r="D56" s="18"/>
-      <x:c r="E56" s="19"/>
-      <x:c r="F56" s="19"/>
-    </x:row>
-    <x:row r="57" ht="28" customHeight="1">
-      <x:c r="A57" s="17"/>
-      <x:c r="B57" s="18"/>
-      <x:c r="C57" s="18"/>
-      <x:c r="D57" s="18"/>
-      <x:c r="E57" s="19"/>
-      <x:c r="F57" s="19"/>
-    </x:row>
-    <x:row r="58" ht="28" customHeight="1">
-      <x:c r="A58" s="17"/>
-      <x:c r="B58" s="18"/>
-      <x:c r="C58" s="18"/>
-      <x:c r="D58" s="18"/>
-      <x:c r="E58" s="19"/>
-      <x:c r="F58" s="19"/>
-    </x:row>
-    <x:row r="59" ht="28" customHeight="1">
-      <x:c r="A59" s="17"/>
-      <x:c r="B59" s="18"/>
-      <x:c r="C59" s="18"/>
-      <x:c r="D59" s="18"/>
-      <x:c r="E59" s="19"/>
-      <x:c r="F59" s="19"/>
-    </x:row>
-    <x:row r="60" ht="28" customHeight="1">
-      <x:c r="A60" s="17"/>
-      <x:c r="B60" s="18"/>
-      <x:c r="C60" s="18"/>
-      <x:c r="D60" s="18"/>
-      <x:c r="E60" s="19"/>
-      <x:c r="F60" s="19"/>
-    </x:row>
-    <x:row r="61" ht="28" customHeight="1">
-      <x:c r="A61" s="17"/>
-      <x:c r="B61" s="18"/>
-      <x:c r="C61" s="18"/>
-      <x:c r="D61" s="18"/>
-      <x:c r="E61" s="19"/>
-      <x:c r="F61" s="19"/>
-    </x:row>
-    <x:row r="62" ht="28" customHeight="1">
-      <x:c r="A62" s="17"/>
-      <x:c r="B62" s="18"/>
-      <x:c r="C62" s="18"/>
-      <x:c r="D62" s="18"/>
-      <x:c r="E62" s="19"/>
-      <x:c r="F62" s="19"/>
-    </x:row>
-    <x:row r="63" ht="28" customHeight="1">
-      <x:c r="A63" s="17"/>
-      <x:c r="B63" s="18"/>
-      <x:c r="C63" s="18"/>
-      <x:c r="D63" s="18"/>
-      <x:c r="E63" s="19"/>
-      <x:c r="F63" s="19"/>
-    </x:row>
-    <x:row r="64" ht="28" customHeight="1">
-      <x:c r="A64" s="17"/>
-      <x:c r="B64" s="18"/>
-      <x:c r="C64" s="18"/>
-      <x:c r="D64" s="18"/>
-      <x:c r="E64" s="19"/>
-      <x:c r="F64" s="19"/>
-    </x:row>
-    <x:row r="65" ht="28" customHeight="1">
-      <x:c r="A65" s="17"/>
-      <x:c r="B65" s="18"/>
-      <x:c r="C65" s="18"/>
-      <x:c r="D65" s="18"/>
-      <x:c r="E65" s="19"/>
-      <x:c r="F65" s="19"/>
-    </x:row>
-    <x:row r="66" ht="28" customHeight="1">
-      <x:c r="A66" s="17"/>
-      <x:c r="B66" s="18"/>
-      <x:c r="C66" s="18"/>
-      <x:c r="D66" s="18"/>
-      <x:c r="E66" s="19"/>
-      <x:c r="F66" s="19"/>
-    </x:row>
-    <x:row r="67" ht="28" customHeight="1">
-      <x:c r="A67" s="17"/>
-      <x:c r="B67" s="18"/>
-      <x:c r="C67" s="18"/>
-      <x:c r="D67" s="18"/>
-      <x:c r="E67" s="19"/>
-      <x:c r="F67" s="19"/>
-    </x:row>
-    <x:row r="68" ht="28" customHeight="1">
-      <x:c r="A68" s="17"/>
-      <x:c r="B68" s="18"/>
-      <x:c r="C68" s="18"/>
-      <x:c r="D68" s="18"/>
-      <x:c r="E68" s="19"/>
-      <x:c r="F68" s="19"/>
-    </x:row>
-    <x:row r="69" ht="28" customHeight="1">
-      <x:c r="A69" s="20"/>
-      <x:c r="B69" s="21"/>
-      <x:c r="C69" s="21"/>
-      <x:c r="D69" s="21"/>
-      <x:c r="E69" s="22"/>
-      <x:c r="F69" s="22"/>
+    <x:row r="20" ht="15" customHeight="1">
+      <x:c r="A20" s="18"/>
+      <x:c r="B20" s="19"/>
+      <x:c r="C20" s="19"/>
+      <x:c r="D20" s="19"/>
+      <x:c r="E20" s="20"/>
+      <x:c r="F20" s="20"/>
+    </x:row>
+    <x:row r="21" ht="15" customHeight="1">
+      <x:c r="A21" s="18"/>
+      <x:c r="B21" s="19"/>
+      <x:c r="C21" s="19"/>
+      <x:c r="D21" s="19"/>
+      <x:c r="E21" s="20"/>
+      <x:c r="F21" s="20"/>
+    </x:row>
+    <x:row r="22" ht="15" customHeight="1">
+      <x:c r="A22" s="18"/>
+      <x:c r="B22" s="19"/>
+      <x:c r="C22" s="19"/>
+      <x:c r="D22" s="19"/>
+      <x:c r="E22" s="20"/>
+      <x:c r="F22" s="20"/>
+    </x:row>
+    <x:row r="23" ht="15" customHeight="1">
+      <x:c r="A23" s="18"/>
+      <x:c r="B23" s="19"/>
+      <x:c r="C23" s="19"/>
+      <x:c r="D23" s="19"/>
+      <x:c r="E23" s="20"/>
+      <x:c r="F23" s="20"/>
+    </x:row>
+    <x:row r="24" ht="15" customHeight="1">
+      <x:c r="A24" s="18"/>
+      <x:c r="B24" s="19"/>
+      <x:c r="C24" s="19"/>
+      <x:c r="D24" s="19"/>
+      <x:c r="E24" s="20"/>
+      <x:c r="F24" s="20"/>
+    </x:row>
+    <x:row r="25" ht="15" customHeight="1">
+      <x:c r="A25" s="18"/>
+      <x:c r="B25" s="19"/>
+      <x:c r="C25" s="19"/>
+      <x:c r="D25" s="19"/>
+      <x:c r="E25" s="20"/>
+      <x:c r="F25" s="20"/>
+    </x:row>
+    <x:row r="26" ht="15" customHeight="1">
+      <x:c r="A26" s="18"/>
+      <x:c r="B26" s="19"/>
+      <x:c r="C26" s="19"/>
+      <x:c r="D26" s="19"/>
+      <x:c r="E26" s="20"/>
+      <x:c r="F26" s="20"/>
+    </x:row>
+    <x:row r="27" ht="15" customHeight="1">
+      <x:c r="A27" s="18"/>
+      <x:c r="B27" s="19"/>
+      <x:c r="C27" s="19"/>
+      <x:c r="D27" s="19"/>
+      <x:c r="E27" s="20"/>
+      <x:c r="F27" s="20"/>
+    </x:row>
+    <x:row r="28" ht="15" customHeight="1">
+      <x:c r="A28" s="18"/>
+      <x:c r="B28" s="19"/>
+      <x:c r="C28" s="19"/>
+      <x:c r="D28" s="19"/>
+      <x:c r="E28" s="20"/>
+      <x:c r="F28" s="20"/>
+    </x:row>
+    <x:row r="29" ht="15" customHeight="1">
+      <x:c r="A29" s="18"/>
+      <x:c r="B29" s="19"/>
+      <x:c r="C29" s="19"/>
+      <x:c r="D29" s="19"/>
+      <x:c r="E29" s="20"/>
+      <x:c r="F29" s="20"/>
+    </x:row>
+    <x:row r="30" ht="15" customHeight="1">
+      <x:c r="A30" s="18"/>
+      <x:c r="B30" s="19"/>
+      <x:c r="C30" s="19"/>
+      <x:c r="D30" s="19"/>
+      <x:c r="E30" s="20"/>
+      <x:c r="F30" s="20"/>
+    </x:row>
+    <x:row r="31" ht="15" customHeight="1">
+      <x:c r="A31" s="18"/>
+      <x:c r="B31" s="19"/>
+      <x:c r="C31" s="19"/>
+      <x:c r="D31" s="19"/>
+      <x:c r="E31" s="20"/>
+      <x:c r="F31" s="20"/>
+    </x:row>
+    <x:row r="32" ht="15" customHeight="1">
+      <x:c r="A32" s="18"/>
+      <x:c r="B32" s="19"/>
+      <x:c r="C32" s="19"/>
+      <x:c r="D32" s="19"/>
+      <x:c r="E32" s="20"/>
+      <x:c r="F32" s="20"/>
+    </x:row>
+    <x:row r="33" ht="15" customHeight="1">
+      <x:c r="A33" s="18"/>
+      <x:c r="B33" s="19"/>
+      <x:c r="C33" s="19"/>
+      <x:c r="D33" s="19"/>
+      <x:c r="E33" s="20"/>
+      <x:c r="F33" s="20"/>
+    </x:row>
+    <x:row r="34" ht="15" customHeight="1">
+      <x:c r="A34" s="18"/>
+      <x:c r="B34" s="19"/>
+      <x:c r="C34" s="19"/>
+      <x:c r="D34" s="19"/>
+      <x:c r="E34" s="20"/>
+      <x:c r="F34" s="20"/>
+    </x:row>
+    <x:row r="35" ht="15" customHeight="1">
+      <x:c r="A35" s="18"/>
+      <x:c r="B35" s="19"/>
+      <x:c r="C35" s="19"/>
+      <x:c r="D35" s="19"/>
+      <x:c r="E35" s="20"/>
+      <x:c r="F35" s="20"/>
+    </x:row>
+    <x:row r="36" ht="15" customHeight="1">
+      <x:c r="A36" s="18"/>
+      <x:c r="B36" s="19"/>
+      <x:c r="C36" s="19"/>
+      <x:c r="D36" s="19"/>
+      <x:c r="E36" s="20"/>
+      <x:c r="F36" s="20"/>
+    </x:row>
+    <x:row r="37" ht="15" customHeight="1">
+      <x:c r="A37" s="18"/>
+      <x:c r="B37" s="19"/>
+      <x:c r="C37" s="19"/>
+      <x:c r="D37" s="19"/>
+      <x:c r="E37" s="20"/>
+      <x:c r="F37" s="20"/>
+    </x:row>
+    <x:row r="38" ht="15" customHeight="1">
+      <x:c r="A38" s="18"/>
+      <x:c r="B38" s="19"/>
+      <x:c r="C38" s="19"/>
+      <x:c r="D38" s="19"/>
+      <x:c r="E38" s="20"/>
+      <x:c r="F38" s="20"/>
+    </x:row>
+    <x:row r="39" ht="15" customHeight="1">
+      <x:c r="A39" s="18"/>
+      <x:c r="B39" s="19"/>
+      <x:c r="C39" s="19"/>
+      <x:c r="D39" s="19"/>
+      <x:c r="E39" s="20"/>
+      <x:c r="F39" s="20"/>
+    </x:row>
+    <x:row r="40" ht="15" customHeight="1">
+      <x:c r="A40" s="18"/>
+      <x:c r="B40" s="19"/>
+      <x:c r="C40" s="19"/>
+      <x:c r="D40" s="19"/>
+      <x:c r="E40" s="20"/>
+      <x:c r="F40" s="20"/>
+    </x:row>
+    <x:row r="41" ht="15" customHeight="1">
+      <x:c r="A41" s="18"/>
+      <x:c r="B41" s="19"/>
+      <x:c r="C41" s="19"/>
+      <x:c r="D41" s="19"/>
+      <x:c r="E41" s="20"/>
+      <x:c r="F41" s="20"/>
+    </x:row>
+    <x:row r="42" ht="15" customHeight="1">
+      <x:c r="A42" s="18"/>
+      <x:c r="B42" s="19"/>
+      <x:c r="C42" s="19"/>
+      <x:c r="D42" s="19"/>
+      <x:c r="E42" s="20"/>
+      <x:c r="F42" s="20"/>
+    </x:row>
+    <x:row r="43" ht="15" customHeight="1">
+      <x:c r="A43" s="18"/>
+      <x:c r="B43" s="19"/>
+      <x:c r="C43" s="19"/>
+      <x:c r="D43" s="19"/>
+      <x:c r="E43" s="20"/>
+      <x:c r="F43" s="20"/>
+    </x:row>
+    <x:row r="44" ht="15" customHeight="1">
+      <x:c r="A44" s="18"/>
+      <x:c r="B44" s="19"/>
+      <x:c r="C44" s="19"/>
+      <x:c r="D44" s="19"/>
+      <x:c r="E44" s="20"/>
+      <x:c r="F44" s="20"/>
+    </x:row>
+    <x:row r="45" ht="15" customHeight="1">
+      <x:c r="A45" s="18"/>
+      <x:c r="B45" s="19"/>
+      <x:c r="C45" s="19"/>
+      <x:c r="D45" s="19"/>
+      <x:c r="E45" s="20"/>
+      <x:c r="F45" s="20"/>
+    </x:row>
+    <x:row r="46" ht="15" customHeight="1">
+      <x:c r="A46" s="18"/>
+      <x:c r="B46" s="19"/>
+      <x:c r="C46" s="19"/>
+      <x:c r="D46" s="19"/>
+      <x:c r="E46" s="20"/>
+      <x:c r="F46" s="20"/>
+    </x:row>
+    <x:row r="47" ht="15" customHeight="1">
+      <x:c r="A47" s="18"/>
+      <x:c r="B47" s="19"/>
+      <x:c r="C47" s="19"/>
+      <x:c r="D47" s="19"/>
+      <x:c r="E47" s="20"/>
+      <x:c r="F47" s="20"/>
+    </x:row>
+    <x:row r="48" ht="15" customHeight="1">
+      <x:c r="A48" s="18"/>
+      <x:c r="B48" s="19"/>
+      <x:c r="C48" s="19"/>
+      <x:c r="D48" s="19"/>
+      <x:c r="E48" s="20"/>
+      <x:c r="F48" s="20"/>
+    </x:row>
+    <x:row r="49" ht="15" customHeight="1">
+      <x:c r="A49" s="18"/>
+      <x:c r="B49" s="19"/>
+      <x:c r="C49" s="19"/>
+      <x:c r="D49" s="19"/>
+      <x:c r="E49" s="20"/>
+      <x:c r="F49" s="20"/>
+    </x:row>
+    <x:row r="50" ht="15" customHeight="1">
+      <x:c r="A50" s="18"/>
+      <x:c r="B50" s="19"/>
+      <x:c r="C50" s="19"/>
+      <x:c r="D50" s="19"/>
+      <x:c r="E50" s="20"/>
+      <x:c r="F50" s="20"/>
+    </x:row>
+    <x:row r="51" ht="15" customHeight="1">
+      <x:c r="A51" s="18"/>
+      <x:c r="B51" s="19"/>
+      <x:c r="C51" s="19"/>
+      <x:c r="D51" s="19"/>
+      <x:c r="E51" s="20"/>
+      <x:c r="F51" s="20"/>
+    </x:row>
+    <x:row r="52" ht="15" customHeight="1">
+      <x:c r="A52" s="18"/>
+      <x:c r="B52" s="19"/>
+      <x:c r="C52" s="19"/>
+      <x:c r="D52" s="19"/>
+      <x:c r="E52" s="20"/>
+      <x:c r="F52" s="20"/>
+    </x:row>
+    <x:row r="53" ht="15" customHeight="1">
+      <x:c r="A53" s="18"/>
+      <x:c r="B53" s="19"/>
+      <x:c r="C53" s="19"/>
+      <x:c r="D53" s="19"/>
+      <x:c r="E53" s="20"/>
+      <x:c r="F53" s="20"/>
+    </x:row>
+    <x:row r="54" ht="15" customHeight="1">
+      <x:c r="A54" s="18"/>
+      <x:c r="B54" s="19"/>
+      <x:c r="C54" s="19"/>
+      <x:c r="D54" s="19"/>
+      <x:c r="E54" s="20"/>
+      <x:c r="F54" s="20"/>
+    </x:row>
+    <x:row r="55" ht="15" customHeight="1">
+      <x:c r="A55" s="18"/>
+      <x:c r="B55" s="19"/>
+      <x:c r="C55" s="19"/>
+      <x:c r="D55" s="19"/>
+      <x:c r="E55" s="20"/>
+      <x:c r="F55" s="20"/>
+    </x:row>
+    <x:row r="56" ht="15" customHeight="1">
+      <x:c r="A56" s="18"/>
+      <x:c r="B56" s="19"/>
+      <x:c r="C56" s="19"/>
+      <x:c r="D56" s="19"/>
+      <x:c r="E56" s="20"/>
+      <x:c r="F56" s="20"/>
+    </x:row>
+    <x:row r="57" ht="15" customHeight="1">
+      <x:c r="A57" s="18"/>
+      <x:c r="B57" s="19"/>
+      <x:c r="C57" s="19"/>
+      <x:c r="D57" s="19"/>
+      <x:c r="E57" s="20"/>
+      <x:c r="F57" s="20"/>
+    </x:row>
+    <x:row r="58" ht="15" customHeight="1">
+      <x:c r="A58" s="18"/>
+      <x:c r="B58" s="19"/>
+      <x:c r="C58" s="19"/>
+      <x:c r="D58" s="19"/>
+      <x:c r="E58" s="20"/>
+      <x:c r="F58" s="20"/>
+    </x:row>
+    <x:row r="59" ht="15" customHeight="1">
+      <x:c r="A59" s="18"/>
+      <x:c r="B59" s="19"/>
+      <x:c r="C59" s="19"/>
+      <x:c r="D59" s="19"/>
+      <x:c r="E59" s="20"/>
+      <x:c r="F59" s="20"/>
+    </x:row>
+    <x:row r="60" ht="15" customHeight="1">
+      <x:c r="A60" s="18"/>
+      <x:c r="B60" s="19"/>
+      <x:c r="C60" s="19"/>
+      <x:c r="D60" s="19"/>
+      <x:c r="E60" s="20"/>
+      <x:c r="F60" s="20"/>
+    </x:row>
+    <x:row r="61" ht="15" customHeight="1">
+      <x:c r="A61" s="18"/>
+      <x:c r="B61" s="19"/>
+      <x:c r="C61" s="19"/>
+      <x:c r="D61" s="19"/>
+      <x:c r="E61" s="20"/>
+      <x:c r="F61" s="20"/>
+    </x:row>
+    <x:row r="62" ht="15" customHeight="1">
+      <x:c r="A62" s="18"/>
+      <x:c r="B62" s="19"/>
+      <x:c r="C62" s="19"/>
+      <x:c r="D62" s="19"/>
+      <x:c r="E62" s="20"/>
+      <x:c r="F62" s="20"/>
+    </x:row>
+    <x:row r="63" ht="15" customHeight="1">
+      <x:c r="A63" s="18"/>
+      <x:c r="B63" s="19"/>
+      <x:c r="C63" s="19"/>
+      <x:c r="D63" s="19"/>
+      <x:c r="E63" s="20"/>
+      <x:c r="F63" s="20"/>
+    </x:row>
+    <x:row r="64" ht="15" customHeight="1">
+      <x:c r="A64" s="18"/>
+      <x:c r="B64" s="19"/>
+      <x:c r="C64" s="19"/>
+      <x:c r="D64" s="19"/>
+      <x:c r="E64" s="20"/>
+      <x:c r="F64" s="20"/>
+    </x:row>
+    <x:row r="65" ht="15" customHeight="1">
+      <x:c r="A65" s="18"/>
+      <x:c r="B65" s="19"/>
+      <x:c r="C65" s="19"/>
+      <x:c r="D65" s="19"/>
+      <x:c r="E65" s="20"/>
+      <x:c r="F65" s="20"/>
+    </x:row>
+    <x:row r="66" ht="15" customHeight="1">
+      <x:c r="A66" s="18"/>
+      <x:c r="B66" s="19"/>
+      <x:c r="C66" s="19"/>
+      <x:c r="D66" s="19"/>
+      <x:c r="E66" s="20"/>
+      <x:c r="F66" s="20"/>
+    </x:row>
+    <x:row r="67" ht="15" customHeight="1">
+      <x:c r="A67" s="18"/>
+      <x:c r="B67" s="19"/>
+      <x:c r="C67" s="19"/>
+      <x:c r="D67" s="19"/>
+      <x:c r="E67" s="20"/>
+      <x:c r="F67" s="20"/>
+    </x:row>
+    <x:row r="68" ht="15" customHeight="1">
+      <x:c r="A68" s="18"/>
+      <x:c r="B68" s="19"/>
+      <x:c r="C68" s="19"/>
+      <x:c r="D68" s="19"/>
+      <x:c r="E68" s="20"/>
+      <x:c r="F68" s="20"/>
+    </x:row>
+    <x:row r="69" ht="15" customHeight="1">
+      <x:c r="A69" s="18"/>
+      <x:c r="B69" s="19"/>
+      <x:c r="C69" s="19"/>
+      <x:c r="D69" s="19"/>
+      <x:c r="E69" s="20"/>
+      <x:c r="F69" s="20"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1105,9 +1095,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19f3c70271984713"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7341d10aeb5b4558"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb07712a5d3cc43b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdbe0f37b90b4595"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1223,7 +1213,7 @@
       <x:c r="A12" s="6" t="str">
         <x:v>Frecuencia (MHz)</x:v>
       </x:c>
-      <x:c r="B12" s="26" t="n">
+      <x:c r="B12" s="24" t="n">
         <x:v>145.5</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
@@ -1234,7 +1224,7 @@
       <x:c r="A13" s="6" t="str">
         <x:v>ROE leída</x:v>
       </x:c>
-      <x:c r="B13" s="27" t="n">
+      <x:c r="B13" s="25" t="n">
         <x:v>1.4</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
@@ -1245,7 +1235,7 @@
       <x:c r="A14" s="6" t="str">
         <x:v>Cable (metros)</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="n">
+      <x:c r="B14" s="25" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="4" t="str">
@@ -1405,6 +1395,6 @@
     <x:mergeCell ref="A31:C31"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b16335f6ac44e1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b708863248841ee"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Preparar ficha de antena para imprimir en carta
</commit_message>
<xml_diff>
--- a/site/assets/docs/ficha-medicion-antena-rufcom.xlsx
+++ b/site/assets/docs/ficha-medicion-antena-rufcom.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi prueba" sheetId="1" r:id="Rce631ae0a75a4d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo y ayuda" sheetId="2" r:id="R546b752d338545fd"/>
+    <x:sheet name="Mi prueba" sheetId="1" r:id="Rce631ae0a75a4d3c"/>
+    <x:sheet name="Ejemplo y ayuda" sheetId="2" r:id="R546b752d338545fd"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Mi prueba'!$A$1:INDEX('Mi prueba'!$F:$F,MAX(39,IFERROR(LOOKUP(2,1/((('Mi prueba'!$A$20:$A$69&lt;&gt;"")+('Mi prueba'!$B$20:$B$69&lt;&gt;"")+('Mi prueba'!$C$20:$C$69&lt;&gt;"")+('Mi prueba'!$D$20:$D$69&lt;&gt;"")+('Mi prueba'!$E$20:$E$69&lt;&gt;"")+('Mi prueba'!$F$20:$F$69&lt;&gt;""))&gt;0),ROW('Mi prueba'!$A$20:$A$69)),20)))</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="0">'Mi prueba'!$1:$19</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="1">'Ejemplo y ayuda'!$A$1:$C$31</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="1">'Ejemplo y ayuda'!$1:$4</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -186,7 +192,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -197,19 +203,21 @@
     <xdr:ext cx="1714500" cy="571500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="06bcd0a7-42ad-4d4c-bb28-a4132ee9dc48"/>
+        <xdr:cNvPr id="1" name="06bcd0a7-42ad-4d4c-bb28-a4132ee9dc48">
+          <a:hlinkClick r:id="rIdRufcomWebsite" tooltip="Abrir RUFCOM: https://rufcom.cl"/>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R151702c94ea04d54"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip r:embed="R151702c94ea04d54"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -218,7 +226,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -229,19 +237,21 @@
     <xdr:ext cx="1714500" cy="571500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="07887ead-9b31-42a0-9194-560e70820e46"/>
+        <xdr:cNvPr id="1" name="07887ead-9b31-42a0-9194-560e70820e46">
+          <a:hlinkClick r:id="rIdRufcomWebsite" tooltip="Abrir RUFCOM: https://rufcom.cl"/>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb95473afedce489e"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip r:embed="Rb95473afedce489e"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -456,9 +466,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF44250A"/>
+    <x:pageSetUpPr fitToPage="1"/>
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1094,18 +1105,24 @@
       <x:formula1>"Antes del cable, desde la radio,En el conector de la antena,Otro punto (explicar en Montaje y lugar)"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7341d10aeb5b4558"/>
+  <x:printOptions horizontalCentered="1" gridLines="0" headings="0"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.4" header="0.15" footer="0.2"/>
+  <x:pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="0" useFirstPageNumber="1" firstPageNumber="1"/>
+  <x:headerFooter>
+    <x:oddFooter>&amp;CRUFCOM · Página &amp;P de &amp;N</x:oddFooter>
+  </x:headerFooter>
+  <x:drawing r:id="R7341d10aeb5b4558"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdbe0f37b90b4595"/>
+    <x:tablePart r:id="Rcdbe0f37b90b4595"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF44250A"/>
+    <x:pageSetUpPr fitToPage="1"/>
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1394,7 +1411,12 @@
     <x:mergeCell ref="A30:C30"/>
     <x:mergeCell ref="A31:C31"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b708863248841ee"/>
+  <x:printOptions horizontalCentered="1" gridLines="0" headings="0"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.4" header="0.15" footer="0.2"/>
+  <x:pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="0" useFirstPageNumber="1" firstPageNumber="1"/>
+  <x:headerFooter>
+    <x:oddFooter>&amp;CRUFCOM · Página &amp;P de &amp;N</x:oddFooter>
+  </x:headerFooter>
+  <x:drawing r:id="R5b708863248841ee"/>
 </x:worksheet>
 </file>
</xml_diff>